<commit_message>
docs: full sync from orderflow/docs - v1.38.16
- Remove legacy/obsolete docs (HR, RealState, capital-humano, old plans)
- Update ROADMAP, CHANGELOG, featurelist for OmniGastro
- Add new audit docs, troubleshooting, timelines
- Sync all current documentation structure
</commit_message>
<xml_diff>
--- a/orderflow/docs/plans/forcaDevendasB2B/Presupuesto_Sistema_B2B.xlsx
+++ b/orderflow/docs/plans/forcaDevendasB2B/Presupuesto_Sistema_B2B.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma" sheetId="1" state="visible" r:id="rId3"/>
@@ -240,11 +240,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="\$#,##0"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="\$#,##0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -402,88 +401,92 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -567,34 +570,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -740,669 +743,669 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E39"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="72.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="5" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="5" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="5" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="5" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="5" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="5" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="5" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="5" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="5" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="5" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="5" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="5" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" s="5" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="5" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" s="5" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="5" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="5" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" s="5" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" s="5" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" s="5" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="E28" s="5" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E30" s="4" t="n">
+      <c r="E30" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="E31" s="5" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="E32" s="5" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" s="5" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E34" s="4" t="n">
+      <c r="E34" s="5" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D35" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="E35" s="5" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D36" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="E36" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D37" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E37" s="4" t="n">
+      <c r="E37" s="5" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="D38" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="E38" s="5" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
-      <c r="C39" s="6" t="s">
+      <c r="A39" s="6"/>
+      <c r="B39" s="6"/>
+      <c r="C39" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D39" s="5"/>
-      <c r="E39" s="7" t="n">
+      <c r="D39" s="6"/>
+      <c r="E39" s="8" t="n">
         <f aca="false">SUM(E2:E38)</f>
         <v>436</v>
       </c>
@@ -1424,183 +1427,183 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <f aca="false">SUMIF(Cronograma!D:D,A6,Cronograma!E:E)</f>
         <v>64</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="12" t="n">
         <f aca="false">B6*C6</f>
         <v>1600</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <f aca="false">SUMIF(Cronograma!D:D,A7,Cronograma!E:E)</f>
         <v>10</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="12" t="n">
         <f aca="false">B7*C7</f>
         <v>150</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <f aca="false">SUMIF(Cronograma!D:D,A8,Cronograma!E:E)</f>
         <v>26</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="12" t="n">
         <f aca="false">B8*C8</f>
         <v>520</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <f aca="false">SUMIF(Cronograma!D:D,A9,Cronograma!E:E)</f>
         <v>170</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="12" t="n">
         <f aca="false">B9*C9</f>
         <v>3400</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="5" t="n">
         <f aca="false">SUMIF(Cronograma!D:D,A10,Cronograma!E:E)</f>
         <v>88</v>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <f aca="false">B10*C10</f>
         <v>1584</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="5" t="n">
         <f aca="false">SUMIF(Cronograma!D:D,A11,Cronograma!E:E)</f>
         <v>78</v>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <f aca="false">B11*C11</f>
         <v>1170</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="13" t="n">
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="14" t="n">
         <f aca="false">SUM(D6:D11)</f>
         <v>8424</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="15" t="n">
+      <c r="B14" s="15"/>
+      <c r="C14" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="17" t="n">
         <f aca="false">D12*C14</f>
         <v>842.4</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="19" t="n">
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="20" t="n">
         <f aca="false">D12+D14</f>
         <v>9266.4</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
+      <c r="A17" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>